<commit_message>
Add normalized length table and update pin assignment files
</commit_message>
<xml_diff>
--- a/doc/pin_assign.xlsx
+++ b/doc/pin_assign.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e643ea309c96c6f6/Documents/Development/kicad/rtcl-tp25k-usb3/doc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryuji\OneDrive\Documents\Development\kicad\rtcl-tp25k-usb3\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="147" documentId="11_AD4D066CA252ABDACC1048F6F9D2CE5873EEDF52" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A77B494-8C1B-4C40-BA37-19AA523A31B4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{704F26EB-9FE7-473F-96D3-0C973174CAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,32 +27,8 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
-    <t>ft601_clk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ft601_txe_n    </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ft601_rxf_n    </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ft601_siwu_n   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ft601_wr_n     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ft601_rd_n     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ft601_oe_n     </t>
-  </si>
-  <si>
     <t>ft601_gpio[0]</t>
     <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ft601_gpio[1]</t>
   </si>
   <si>
     <t>ft601_be[0]</t>
@@ -642,6 +618,38 @@
   </si>
   <si>
     <t>FT601_CLK</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_clk</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_txe_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_rxf_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_siwu_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_wr_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_rd_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_oe_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_gpio[1]</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -694,10 +702,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -988,646 +995,646 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18.5" thickBot="1">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>138</v>
+        <v>129</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18.5" thickTop="1">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>176</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="D2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>177</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>178</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>179</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>180</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D6" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>181</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>182</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D11" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="D14" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D20" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D21" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C22" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D22" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D23" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C24" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D24" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C25" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D25" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D26" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B27" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C28" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D28" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B29" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D29" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C30" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D30" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B31" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C32" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C33" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B34" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B35" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C35" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D35" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B36" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C36" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B37" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C37" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B38" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C38" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="D38" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B39" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C39" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="D39" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B40" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C40" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="D40" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B41" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C41" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="D41" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B42" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C42" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="D42" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B43" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="C43" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D43" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B44" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="D44" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B45" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C45" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="D45" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="B46" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="C46" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="D46" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor KiCad project files for improved layout and organization
- Updated active layer in the project file to layer 5 for better visibility.
- Modified selection filter settings to hide dimensions, footprints, graphics, keepouts, other items, pads, tracks, vias, and zones.
- Cleared used designators in the project file to streamline component management.
- Adjusted junction and wire coordinates in the schematic for better alignment and clarity.
- Renamed labels in the schematic for consistency and clarity.
- Updated component positions and properties in the schematic to enhance layout.
- Modified footprint properties in the module file for improved design accuracy.
- Changed UUIDs for various elements to ensure uniqueness and prevent conflicts.
</commit_message>
<xml_diff>
--- a/doc/pin_assign.xlsx
+++ b/doc/pin_assign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e643ea309c96c6f6/Documents/Development/kicad/rtcl-tp25k-usb3/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="631" documentId="13_ncr:1_{704F26EB-9FE7-473F-96D3-0C973174CAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7839B63E-99C9-4EAD-9557-C4B5F641D4B1}"/>
+  <xr:revisionPtr revIDLastSave="634" documentId="13_ncr:1_{704F26EB-9FE7-473F-96D3-0C973174CAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BF1F114-A25A-48FC-B7AC-6EF32D47EAE1}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="16080" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="57840" yWindow="13710" windowWidth="26130" windowHeight="17970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -650,624 +650,627 @@
     <t>E11_IOL3A</t>
   </si>
   <si>
+    <t>E3_IOB60A_40P</t>
+  </si>
+  <si>
+    <t>VCCIO6_7</t>
+  </si>
+  <si>
+    <t>H5</t>
+  </si>
+  <si>
+    <t>J5</t>
+  </si>
+  <si>
+    <t>L5</t>
+  </si>
+  <si>
+    <t>K5</t>
+  </si>
+  <si>
+    <t>H8</t>
+  </si>
+  <si>
+    <t>H7</t>
+  </si>
+  <si>
+    <t>G7</t>
+  </si>
+  <si>
+    <t>G8</t>
+  </si>
+  <si>
+    <t>F5</t>
+  </si>
+  <si>
+    <t>G5</t>
+  </si>
+  <si>
+    <t>K11</t>
+  </si>
+  <si>
+    <t>L11</t>
+  </si>
+  <si>
+    <t>E11</t>
+  </si>
+  <si>
+    <t>E10</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>E8</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>L6</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>E3</t>
+  </si>
+  <si>
+    <t>K6</t>
+  </si>
+  <si>
+    <t>K7</t>
+  </si>
+  <si>
+    <t>J7</t>
+  </si>
+  <si>
+    <t>L7</t>
+  </si>
+  <si>
+    <t>L8</t>
+  </si>
+  <si>
+    <t>L10</t>
+  </si>
+  <si>
+    <t>K10</t>
+  </si>
+  <si>
+    <t>L9</t>
+  </si>
+  <si>
+    <t>K9</t>
+  </si>
+  <si>
+    <t>J8</t>
+  </si>
+  <si>
+    <t>K8</t>
+  </si>
+  <si>
+    <t>F7</t>
+  </si>
+  <si>
+    <t>F6</t>
+  </si>
+  <si>
+    <t>J11</t>
+  </si>
+  <si>
+    <t>J10</t>
+  </si>
+  <si>
+    <t>H11</t>
+  </si>
+  <si>
+    <t>H10</t>
+  </si>
+  <si>
+    <t>G11</t>
+  </si>
+  <si>
+    <t>G10</t>
+  </si>
+  <si>
+    <t>D11</t>
+  </si>
+  <si>
+    <t>D10</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>B11</t>
+  </si>
+  <si>
+    <t>B10</t>
+  </si>
+  <si>
+    <t>FPGA</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>NAME</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>bank</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>attr</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Voltage</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A11</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>VCCIO2_3</t>
+  </si>
+  <si>
+    <t>L2_IOR18A_40P</t>
+  </si>
+  <si>
+    <t>G2_IOR24A_40P</t>
+  </si>
+  <si>
+    <t>L3_IOR31B_40P</t>
+  </si>
+  <si>
+    <t>J1_IOR33A_40P</t>
+  </si>
+  <si>
+    <t>J2_IOR33B_40P</t>
+  </si>
+  <si>
+    <t>G4_IOB89A_40P</t>
+  </si>
+  <si>
+    <t>H4_IOB89B_40P</t>
+  </si>
+  <si>
+    <t>H1_IOB91A_40P</t>
+  </si>
+  <si>
+    <t>H2_IOB91B_40P</t>
+  </si>
+  <si>
+    <t>1.8V</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2.5V</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>3.3V</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>5V</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>L2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>G2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>L3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>J1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>J2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>G4</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>H4</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>H1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>H2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C2_IOB4B_40P</t>
+  </si>
+  <si>
+    <t>F2_IOB26A_40P</t>
+  </si>
+  <si>
+    <t>F1_IOB26B_40P</t>
+  </si>
+  <si>
+    <t>A1_IOB24A_40P</t>
+  </si>
+  <si>
+    <t>E1_IOB12B_40P</t>
+  </si>
+  <si>
+    <t>D1_IOB14B_40P</t>
+  </si>
+  <si>
+    <t>B2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>F2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>F1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>D8</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>E1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>D1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>RPLL</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C1_JTAG_TCK</t>
+  </si>
+  <si>
+    <t>B1_JTAG_TMS</t>
+  </si>
+  <si>
+    <t>A2_JTAG_TDO</t>
+  </si>
+  <si>
+    <t>A3_JTAG_TDI</t>
+  </si>
+  <si>
+    <t>M0_D3_P</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_D3_N</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_D2_P</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_D2_N</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_CK_P</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_CK_N</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_D1_P</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_D1_N</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_D0_P</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M0_D0_N</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_reset_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ft601_wakeup</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>FT601_RESET</t>
+  </si>
+  <si>
+    <t>FT601_WAKEUP</t>
+  </si>
+  <si>
+    <t>JTAG</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_ck_p</t>
+  </si>
+  <si>
+    <t>mipi_ck_n</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_d_p[3]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_d_n[3]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_d_p[2]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_d_n[2]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_d_p[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_d_n[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_pwr_en</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_scl</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_sda</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>led[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>E8_READY</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B3_IOB56A_UART_RX</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C3_IOB56B_UART_TX</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>D7_DONE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>D8_RECONFIG</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B2_IOB4A_40P</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>E2</t>
+  </si>
+  <si>
+    <t>IOB12A</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>LOC</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>in_clk50</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>K7_IOT21A_40P</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[2]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[3]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[4]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[5]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[7]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>pmod[6]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_gpio[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mipi_gpio[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>led[1]</t>
+  </si>
+  <si>
+    <t>led[2]</t>
+  </si>
+  <si>
+    <t>led[3]</t>
+  </si>
+  <si>
+    <t>push_sw[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>push_sw[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>dip_sw[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>dip_sw[1]</t>
+  </si>
+  <si>
+    <t>test[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>test[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A5</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B5</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A6</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B6</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A7</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B7</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A8</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B8</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A9</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B9</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B11_IOL12A</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B10_IOL12B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C11_IOL5A</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C10_IOL5B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>E10_IOL3B</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>A11_IOL14A</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>A10_IOL14B</t>
-  </si>
-  <si>
-    <t>E3_IOB60A_40P</t>
-  </si>
-  <si>
-    <t>VCCIO6_7</t>
-  </si>
-  <si>
-    <t>H5</t>
-  </si>
-  <si>
-    <t>J5</t>
-  </si>
-  <si>
-    <t>L5</t>
-  </si>
-  <si>
-    <t>K5</t>
-  </si>
-  <si>
-    <t>H8</t>
-  </si>
-  <si>
-    <t>H7</t>
-  </si>
-  <si>
-    <t>G7</t>
-  </si>
-  <si>
-    <t>G8</t>
-  </si>
-  <si>
-    <t>F5</t>
-  </si>
-  <si>
-    <t>G5</t>
-  </si>
-  <si>
-    <t>K11</t>
-  </si>
-  <si>
-    <t>L11</t>
-  </si>
-  <si>
-    <t>E11</t>
-  </si>
-  <si>
-    <t>E10</t>
-  </si>
-  <si>
-    <t>A10</t>
-  </si>
-  <si>
-    <t>E8</t>
-  </si>
-  <si>
-    <t>D7</t>
-  </si>
-  <si>
-    <t>L6</t>
-  </si>
-  <si>
-    <t>B3</t>
-  </si>
-  <si>
-    <t>C3</t>
-  </si>
-  <si>
-    <t>E3</t>
-  </si>
-  <si>
-    <t>K6</t>
-  </si>
-  <si>
-    <t>K7</t>
-  </si>
-  <si>
-    <t>J7</t>
-  </si>
-  <si>
-    <t>L7</t>
-  </si>
-  <si>
-    <t>L8</t>
-  </si>
-  <si>
-    <t>L10</t>
-  </si>
-  <si>
-    <t>K10</t>
-  </si>
-  <si>
-    <t>L9</t>
-  </si>
-  <si>
-    <t>K9</t>
-  </si>
-  <si>
-    <t>J8</t>
-  </si>
-  <si>
-    <t>K8</t>
-  </si>
-  <si>
-    <t>F7</t>
-  </si>
-  <si>
-    <t>F6</t>
-  </si>
-  <si>
-    <t>J11</t>
-  </si>
-  <si>
-    <t>J10</t>
-  </si>
-  <si>
-    <t>H11</t>
-  </si>
-  <si>
-    <t>H10</t>
-  </si>
-  <si>
-    <t>G11</t>
-  </si>
-  <si>
-    <t>G10</t>
-  </si>
-  <si>
-    <t>D11</t>
-  </si>
-  <si>
-    <t>D10</t>
-  </si>
-  <si>
-    <t>C11</t>
-  </si>
-  <si>
-    <t>C10</t>
-  </si>
-  <si>
-    <t>B11</t>
-  </si>
-  <si>
-    <t>B10</t>
-  </si>
-  <si>
-    <t>FPGA</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>NAME</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>bank</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>attr</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Voltage</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A11</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>VCCIO2_3</t>
-  </si>
-  <si>
-    <t>L2_IOR18A_40P</t>
-  </si>
-  <si>
-    <t>G2_IOR24A_40P</t>
-  </si>
-  <si>
-    <t>L3_IOR31B_40P</t>
-  </si>
-  <si>
-    <t>J1_IOR33A_40P</t>
-  </si>
-  <si>
-    <t>J2_IOR33B_40P</t>
-  </si>
-  <si>
-    <t>G4_IOB89A_40P</t>
-  </si>
-  <si>
-    <t>H4_IOB89B_40P</t>
-  </si>
-  <si>
-    <t>H1_IOB91A_40P</t>
-  </si>
-  <si>
-    <t>H2_IOB91B_40P</t>
-  </si>
-  <si>
-    <t>1.8V</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2.5V</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>3.3V</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>5V</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>L2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>G2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>L3</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>J1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>J2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>G4</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>H4</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>H1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>H2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C2_IOB4B_40P</t>
-  </si>
-  <si>
-    <t>F2_IOB26A_40P</t>
-  </si>
-  <si>
-    <t>F1_IOB26B_40P</t>
-  </si>
-  <si>
-    <t>A1_IOB24A_40P</t>
-  </si>
-  <si>
-    <t>E1_IOB12B_40P</t>
-  </si>
-  <si>
-    <t>D1_IOB14B_40P</t>
-  </si>
-  <si>
-    <t>B2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>F2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>F1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>D8</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>E1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>D1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>RPLL</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C1_JTAG_TCK</t>
-  </si>
-  <si>
-    <t>B1_JTAG_TMS</t>
-  </si>
-  <si>
-    <t>A2_JTAG_TDO</t>
-  </si>
-  <si>
-    <t>A3_JTAG_TDI</t>
-  </si>
-  <si>
-    <t>M0_D3_P</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_D3_N</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_D2_P</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_D2_N</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_CK_P</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_CK_N</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_D1_P</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_D1_N</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_D0_P</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>M0_D0_N</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A3</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ft601_reset_n</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ft601_wakeup</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>FT601_RESET</t>
-  </si>
-  <si>
-    <t>FT601_WAKEUP</t>
-  </si>
-  <si>
-    <t>JTAG</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_ck_p</t>
-  </si>
-  <si>
-    <t>mipi_ck_n</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_d_p[3]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_d_n[3]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_d_p[2]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_d_n[2]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_d_p[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_d_n[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_pwr_en</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_scl</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_sda</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>led[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>E8_READY</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B3_IOB56A_UART_RX</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C3_IOB56B_UART_TX</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>D7_DONE</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>D8_RECONFIG</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B2_IOB4A_40P</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>E2</t>
-  </si>
-  <si>
-    <t>IOB12A</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>LOC</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>in_clk50</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>K7_IOT21A_40P</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[2]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[3]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[4]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[5]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[7]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>pmod[6]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_gpio[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mipi_gpio[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>led[1]</t>
-  </si>
-  <si>
-    <t>led[2]</t>
-  </si>
-  <si>
-    <t>led[3]</t>
-  </si>
-  <si>
-    <t>push_sw[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>push_sw[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>dip_sw[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>dip_sw[1]</t>
-  </si>
-  <si>
-    <t>test[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>test[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A5</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B5</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A6</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B6</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A7</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B7</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A8</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B8</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A9</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B9</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>No.</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B11_IOL12A</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B10_IOL12B</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C11_IOL5A</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C10_IOL5B</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1363,7 +1366,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1379,9 +1382,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1709,10 +1709,10 @@
         <v>166</v>
       </c>
       <c r="B3" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D3" t="s">
         <v>156</v>
@@ -1793,7 +1793,7 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C9" t="s">
         <v>43</v>
@@ -1807,7 +1807,7 @@
         <v>172</v>
       </c>
       <c r="B10" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C10" t="s">
         <v>44</v>
@@ -1821,10 +1821,10 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C11" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D11" t="s">
         <v>120</v>
@@ -1835,10 +1835,10 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C12" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D12" t="s">
         <v>121</v>
@@ -2297,10 +2297,10 @@
         <v>35</v>
       </c>
       <c r="B45" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C45" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D45" t="s">
         <v>154</v>
@@ -2311,10 +2311,10 @@
         <v>36</v>
       </c>
       <c r="B46" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C46" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D46" t="s">
         <v>155</v>
@@ -2322,30 +2322,30 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B47" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C47" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D47" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B48" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C48" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D48" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -2370,7 +2370,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18.5" thickBot="1">
       <c r="A1" s="7" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>173</v>
@@ -2379,25 +2379,25 @@
         <v>79</v>
       </c>
       <c r="D1" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="J1" s="9" t="s">
-        <v>317</v>
+      <c r="J1" s="8" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.5" thickTop="1">
@@ -2424,7 +2424,7 @@
         <v/>
       </c>
       <c r="J2" s="5" t="str">
-        <f>IF(I2&lt;&gt;"","IO_LOC """&amp;I2&amp;""" "&amp;D2&amp;";", "")</f>
+        <f t="shared" ref="J2:J35" si="0">IF(I2&lt;&gt;"","IO_LOC """&amp;I2&amp;""" "&amp;D2&amp;";", "")</f>
         <v/>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
         <v/>
       </c>
       <c r="J3" s="3" t="str">
-        <f>IF(I3&lt;&gt;"","IO_LOC """&amp;I3&amp;""" "&amp;D3&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
         <v/>
       </c>
       <c r="J4" s="3" t="str">
-        <f>IF(I4&lt;&gt;"","IO_LOC """&amp;I4&amp;""" "&amp;D4&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
         <v/>
       </c>
       <c r="J5" s="3" t="str">
-        <f>IF(I5&lt;&gt;"","IO_LOC """&amp;I5&amp;""" "&amp;D5&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
         <v/>
       </c>
       <c r="J6" s="3" t="str">
-        <f>IF(I6&lt;&gt;"","IO_LOC """&amp;I6&amp;""" "&amp;D6&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2554,7 +2554,7 @@
         <v/>
       </c>
       <c r="J7" s="3" t="str">
-        <f>IF(I7&lt;&gt;"","IO_LOC """&amp;I7&amp;""" "&amp;D7&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
         <v/>
       </c>
       <c r="J8" s="3" t="str">
-        <f>IF(I8&lt;&gt;"","IO_LOC """&amp;I8&amp;""" "&amp;D8&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
         <v/>
       </c>
       <c r="J9" s="3" t="str">
-        <f>IF(I9&lt;&gt;"","IO_LOC """&amp;I9&amp;""" "&amp;D9&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2634,7 +2634,7 @@
         <v/>
       </c>
       <c r="J10" s="3" t="str">
-        <f>IF(I10&lt;&gt;"","IO_LOC """&amp;I10&amp;""" "&amp;D10&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -2660,7 +2660,7 @@
         <v/>
       </c>
       <c r="J11" s="3" t="str">
-        <f>IF(I11&lt;&gt;"","IO_LOC """&amp;I11&amp;""" "&amp;D11&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
@@ -2686,7 +2686,7 @@
         <v/>
       </c>
       <c r="J12" s="3" t="str">
-        <f>IF(I12&lt;&gt;"","IO_LOC """&amp;I12&amp;""" "&amp;D12&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
         <v/>
       </c>
       <c r="J13" s="3" t="str">
-        <f>IF(I13&lt;&gt;"","IO_LOC """&amp;I13&amp;""" "&amp;D13&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v/>
       </c>
       <c r="J14" s="3" t="str">
-        <f>IF(I14&lt;&gt;"","IO_LOC """&amp;I14&amp;""" "&amp;D14&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="J15" s="3" t="str">
-        <f>IF(I15&lt;&gt;"","IO_LOC """&amp;I15&amp;""" "&amp;D15&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -2790,7 +2790,7 @@
         <v/>
       </c>
       <c r="J16" s="3" t="str">
-        <f>IF(I16&lt;&gt;"","IO_LOC """&amp;I16&amp;""" "&amp;D16&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -2816,7 +2816,7 @@
         <v/>
       </c>
       <c r="J17" s="3" t="str">
-        <f>IF(I17&lt;&gt;"","IO_LOC """&amp;I17&amp;""" "&amp;D17&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -2842,7 +2842,7 @@
         <v/>
       </c>
       <c r="J18" s="3" t="str">
-        <f>IF(I18&lt;&gt;"","IO_LOC """&amp;I18&amp;""" "&amp;D18&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -2868,7 +2868,7 @@
         <v/>
       </c>
       <c r="J19" s="3" t="str">
-        <f>IF(I19&lt;&gt;"","IO_LOC """&amp;I19&amp;""" "&amp;D19&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="J20" s="3" t="str">
-        <f>IF(I20&lt;&gt;"","IO_LOC """&amp;I20&amp;""" "&amp;D20&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -2920,7 +2920,7 @@
         <v/>
       </c>
       <c r="J21" s="3" t="str">
-        <f>IF(I21&lt;&gt;"","IO_LOC """&amp;I21&amp;""" "&amp;D21&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -2946,7 +2946,7 @@
         <v/>
       </c>
       <c r="J22" s="3" t="str">
-        <f>IF(I22&lt;&gt;"","IO_LOC """&amp;I22&amp;""" "&amp;D22&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -2972,7 +2972,7 @@
         <v/>
       </c>
       <c r="J23" s="3" t="str">
-        <f>IF(I23&lt;&gt;"","IO_LOC """&amp;I23&amp;""" "&amp;D23&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -2998,7 +2998,7 @@
         <v/>
       </c>
       <c r="J24" s="3" t="str">
-        <f>IF(I24&lt;&gt;"","IO_LOC """&amp;I24&amp;""" "&amp;D24&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -3024,7 +3024,7 @@
         <v/>
       </c>
       <c r="J25" s="3" t="str">
-        <f>IF(I25&lt;&gt;"","IO_LOC """&amp;I25&amp;""" "&amp;D25&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -3050,7 +3050,7 @@
         <v/>
       </c>
       <c r="J26" s="3" t="str">
-        <f>IF(I26&lt;&gt;"","IO_LOC """&amp;I26&amp;""" "&amp;D26&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -3076,7 +3076,7 @@
         <v/>
       </c>
       <c r="J27" s="3" t="str">
-        <f>IF(I27&lt;&gt;"","IO_LOC """&amp;I27&amp;""" "&amp;D27&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3102,7 +3102,7 @@
         <v/>
       </c>
       <c r="J28" s="3" t="str">
-        <f>IF(I28&lt;&gt;"","IO_LOC """&amp;I28&amp;""" "&amp;D28&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
         <v/>
       </c>
       <c r="J29" s="3" t="str">
-        <f>IF(I29&lt;&gt;"","IO_LOC """&amp;I29&amp;""" "&amp;D29&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3143,10 +3143,10 @@
         <v>13</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="F30" s="4">
         <v>5</v>
@@ -3160,7 +3160,7 @@
         <v/>
       </c>
       <c r="J30" s="3" t="str">
-        <f>IF(I30&lt;&gt;"","IO_LOC """&amp;I30&amp;""" "&amp;D30&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
         <v/>
       </c>
       <c r="J31" s="3" t="str">
-        <f>IF(I31&lt;&gt;"","IO_LOC """&amp;I31&amp;""" "&amp;D31&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3212,7 +3212,7 @@
         <v/>
       </c>
       <c r="J32" s="3" t="str">
-        <f>IF(I32&lt;&gt;"","IO_LOC """&amp;I32&amp;""" "&amp;D32&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
         <v/>
       </c>
       <c r="J33" s="3" t="str">
-        <f>IF(I33&lt;&gt;"","IO_LOC """&amp;I33&amp;""" "&amp;D33&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3264,7 +3264,7 @@
         <v/>
       </c>
       <c r="J34" s="3" t="str">
-        <f>IF(I34&lt;&gt;"","IO_LOC """&amp;I34&amp;""" "&amp;D34&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3290,7 +3290,7 @@
         <v/>
       </c>
       <c r="J35" s="3" t="str">
-        <f>IF(I35&lt;&gt;"","IO_LOC """&amp;I35&amp;""" "&amp;D35&amp;";", "")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3328,10 +3328,10 @@
         <v>51</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F37" s="4">
         <v>6</v>
@@ -3341,10 +3341,10 @@
         <v>1.8</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="J37" s="3" t="str">
-        <f>IF(I37&lt;&gt;"","IO_LOC """&amp;I37&amp;""" "&amp;D37&amp;";", "")</f>
+        <f t="shared" ref="J37:J68" si="1">IF(I37&lt;&gt;"","IO_LOC """&amp;I37&amp;""" "&amp;D37&amp;";", "")</f>
         <v>IO_LOC "dip_sw[0]" C11;</v>
       </c>
     </row>
@@ -3359,10 +3359,10 @@
         <v>53</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F38" s="4">
         <v>6</v>
@@ -3372,10 +3372,10 @@
         <v>1.8</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="J38" s="3" t="str">
-        <f>IF(I38&lt;&gt;"","IO_LOC """&amp;I38&amp;""" "&amp;D38&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "dip_sw[1]" C10;</v>
       </c>
     </row>
@@ -3390,10 +3390,10 @@
         <v>26</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F39" s="4">
         <v>2</v>
@@ -3409,7 +3409,7 @@
         <v>ft601_be[0]</v>
       </c>
       <c r="J39" s="3" t="str">
-        <f>IF(I39&lt;&gt;"","IO_LOC """&amp;I39&amp;""" "&amp;D39&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_be[0]" J1;</v>
       </c>
     </row>
@@ -3424,10 +3424,10 @@
         <v>24</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F40" s="4">
         <v>2</v>
@@ -3443,7 +3443,7 @@
         <v>ft601_be[1]</v>
       </c>
       <c r="J40" s="3" t="str">
-        <f>IF(I40&lt;&gt;"","IO_LOC """&amp;I40&amp;""" "&amp;D40&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_be[1]" L3;</v>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
         <v>ft601_be[2]</v>
       </c>
       <c r="J41" s="3" t="str">
-        <f>IF(I41&lt;&gt;"","IO_LOC """&amp;I41&amp;""" "&amp;D41&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_be[2]" L4;</v>
       </c>
     </row>
@@ -3509,7 +3509,7 @@
         <v>ft601_be[3]</v>
       </c>
       <c r="J42" s="3" t="str">
-        <f>IF(I42&lt;&gt;"","IO_LOC """&amp;I42&amp;""" "&amp;D42&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_be[3]" G1;</v>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
         <v>10</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>61</v>
@@ -3543,7 +3543,7 @@
         <v>ft601_clk</v>
       </c>
       <c r="J43" s="3" t="str">
-        <f>IF(I43&lt;&gt;"","IO_LOC """&amp;I43&amp;""" "&amp;D43&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_clk" K5;</v>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
         <v>48</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>45</v>
@@ -3575,7 +3575,7 @@
         <v>ft601_data[0]</v>
       </c>
       <c r="J44" s="3" t="str">
-        <f>IF(I44&lt;&gt;"","IO_LOC """&amp;I44&amp;""" "&amp;D44&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[0]" L11;</v>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
         <v>46</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
@@ -3607,7 +3607,7 @@
         <v>ft601_data[1]</v>
       </c>
       <c r="J45" s="3" t="str">
-        <f>IF(I45&lt;&gt;"","IO_LOC """&amp;I45&amp;""" "&amp;D45&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[1]" K11;</v>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>22</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>55</v>
@@ -3639,7 +3639,7 @@
         <v>ft601_data[10]</v>
       </c>
       <c r="J46" s="3" t="str">
-        <f>IF(I46&lt;&gt;"","IO_LOC """&amp;I46&amp;""" "&amp;D46&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[10]" G5;</v>
       </c>
     </row>
@@ -3654,7 +3654,7 @@
         <v>20</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>56</v>
@@ -3671,7 +3671,7 @@
         <v>ft601_data[11]</v>
       </c>
       <c r="J47" s="3" t="str">
-        <f>IF(I47&lt;&gt;"","IO_LOC """&amp;I47&amp;""" "&amp;D47&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[11]" F5;</v>
       </c>
     </row>
@@ -3686,7 +3686,7 @@
         <v>18</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>57</v>
@@ -3703,7 +3703,7 @@
         <v>ft601_data[12]</v>
       </c>
       <c r="J48" s="3" t="str">
-        <f>IF(I48&lt;&gt;"","IO_LOC """&amp;I48&amp;""" "&amp;D48&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[12]" G8;</v>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
         <v>16</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>58</v>
@@ -3735,7 +3735,7 @@
         <v>ft601_data[13]</v>
       </c>
       <c r="J49" s="3" t="str">
-        <f>IF(I49&lt;&gt;"","IO_LOC """&amp;I49&amp;""" "&amp;D49&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[13]" G7;</v>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
         <v>14</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>59</v>
@@ -3767,7 +3767,7 @@
         <v>ft601_data[14]</v>
       </c>
       <c r="J50" s="3" t="str">
-        <f>IF(I50&lt;&gt;"","IO_LOC """&amp;I50&amp;""" "&amp;D50&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[14]" H7;</v>
       </c>
     </row>
@@ -3782,7 +3782,7 @@
         <v>12</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>60</v>
@@ -3799,7 +3799,7 @@
         <v>ft601_data[15]</v>
       </c>
       <c r="J51" s="3" t="str">
-        <f>IF(I51&lt;&gt;"","IO_LOC """&amp;I51&amp;""" "&amp;D51&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[15]" H8;</v>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
         <v>4</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>62</v>
@@ -3833,7 +3833,7 @@
         <v>ft601_data[16]</v>
       </c>
       <c r="J52" s="3" t="str">
-        <f>IF(I52&lt;&gt;"","IO_LOC """&amp;I52&amp;""" "&amp;D52&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[16]" H5;</v>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
         <v>6</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E53" s="4" t="s">
         <v>63</v>
@@ -3867,7 +3867,7 @@
         <v>ft601_data[17]</v>
       </c>
       <c r="J53" s="3" t="str">
-        <f>IF(I53&lt;&gt;"","IO_LOC """&amp;I53&amp;""" "&amp;D53&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[17]" J5;</v>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
         <v>8</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E54" s="4" t="s">
         <v>64</v>
@@ -3901,7 +3901,7 @@
         <v>ft601_data[18]</v>
       </c>
       <c r="J54" s="3" t="str">
-        <f>IF(I54&lt;&gt;"","IO_LOC """&amp;I54&amp;""" "&amp;D54&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[18]" L5;</v>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
         <v>3</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>65</v>
@@ -3933,7 +3933,7 @@
         <v>ft601_data[19]</v>
       </c>
       <c r="J55" s="3" t="str">
-        <f>IF(I55&lt;&gt;"","IO_LOC """&amp;I55&amp;""" "&amp;D55&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[19]" L9;</v>
       </c>
     </row>
@@ -3948,7 +3948,7 @@
         <v>44</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>47</v>
@@ -3965,7 +3965,7 @@
         <v>ft601_data[2]</v>
       </c>
       <c r="J56" s="3" t="str">
-        <f>IF(I56&lt;&gt;"","IO_LOC """&amp;I56&amp;""" "&amp;D56&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[2]" K10;</v>
       </c>
     </row>
@@ -3980,7 +3980,7 @@
         <v>5</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E57" s="4" t="s">
         <v>66</v>
@@ -3997,7 +3997,7 @@
         <v>ft601_data[20]</v>
       </c>
       <c r="J57" s="3" t="str">
-        <f>IF(I57&lt;&gt;"","IO_LOC """&amp;I57&amp;""" "&amp;D57&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[20]" K9;</v>
       </c>
     </row>
@@ -4012,7 +4012,7 @@
         <v>7</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E58" s="4" t="s">
         <v>67</v>
@@ -4031,7 +4031,7 @@
         <v>ft601_data[21]</v>
       </c>
       <c r="J58" s="3" t="str">
-        <f>IF(I58&lt;&gt;"","IO_LOC """&amp;I58&amp;""" "&amp;D58&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[21]" J8;</v>
       </c>
     </row>
@@ -4046,7 +4046,7 @@
         <v>9</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E59" s="4" t="s">
         <v>68</v>
@@ -4065,7 +4065,7 @@
         <v>ft601_data[22]</v>
       </c>
       <c r="J59" s="3" t="str">
-        <f>IF(I59&lt;&gt;"","IO_LOC """&amp;I59&amp;""" "&amp;D59&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[22]" K8;</v>
       </c>
     </row>
@@ -4080,7 +4080,7 @@
         <v>11</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E60" s="4" t="s">
         <v>69</v>
@@ -4099,7 +4099,7 @@
         <v>ft601_data[23]</v>
       </c>
       <c r="J60" s="3" t="str">
-        <f>IF(I60&lt;&gt;"","IO_LOC """&amp;I60&amp;""" "&amp;D60&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[23]" F7;</v>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
         <v>13</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>70</v>
@@ -4131,7 +4131,7 @@
         <v>ft601_data[24]</v>
       </c>
       <c r="J61" s="3" t="str">
-        <f>IF(I61&lt;&gt;"","IO_LOC """&amp;I61&amp;""" "&amp;D61&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[24]" F6;</v>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
         <v>33</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>71</v>
@@ -4165,7 +4165,7 @@
         <v>ft601_data[25]</v>
       </c>
       <c r="J62" s="3" t="str">
-        <f>IF(I62&lt;&gt;"","IO_LOC """&amp;I62&amp;""" "&amp;D62&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[25]" J11;</v>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
         <v>35</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E63" s="4" t="s">
         <v>72</v>
@@ -4199,7 +4199,7 @@
         <v>ft601_data[26]</v>
       </c>
       <c r="J63" s="3" t="str">
-        <f>IF(I63&lt;&gt;"","IO_LOC """&amp;I63&amp;""" "&amp;D63&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[26]" J10;</v>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
         <v>37</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>73</v>
@@ -4233,7 +4233,7 @@
         <v>ft601_data[27]</v>
       </c>
       <c r="J64" s="3" t="str">
-        <f>IF(I64&lt;&gt;"","IO_LOC """&amp;I64&amp;""" "&amp;D64&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[27]" H11;</v>
       </c>
     </row>
@@ -4248,7 +4248,7 @@
         <v>39</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E65" s="4" t="s">
         <v>74</v>
@@ -4267,7 +4267,7 @@
         <v>ft601_data[28]</v>
       </c>
       <c r="J65" s="3" t="str">
-        <f>IF(I65&lt;&gt;"","IO_LOC """&amp;I65&amp;""" "&amp;D65&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[28]" H10;</v>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
         <v>41</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E66" s="4" t="s">
         <v>75</v>
@@ -4299,7 +4299,7 @@
         <v>ft601_data[29]</v>
       </c>
       <c r="J66" s="3" t="str">
-        <f>IF(I66&lt;&gt;"","IO_LOC """&amp;I66&amp;""" "&amp;D66&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[29]" G11;</v>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
         <v>42</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>48</v>
@@ -4331,7 +4331,7 @@
         <v>ft601_data[3]</v>
       </c>
       <c r="J67" s="3" t="str">
-        <f>IF(I67&lt;&gt;"","IO_LOC """&amp;I67&amp;""" "&amp;D67&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[3]" L10;</v>
       </c>
     </row>
@@ -4346,10 +4346,10 @@
         <v>30</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F68" s="4">
         <v>3</v>
@@ -4365,7 +4365,7 @@
         <v>ft601_data[30]</v>
       </c>
       <c r="J68" s="3" t="str">
-        <f>IF(I68&lt;&gt;"","IO_LOC """&amp;I68&amp;""" "&amp;D68&amp;";", "")</f>
+        <f t="shared" si="1"/>
         <v>IO_LOC "ft601_data[30]" G4;</v>
       </c>
     </row>
@@ -4380,10 +4380,10 @@
         <v>28</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="F69" s="4">
         <v>2</v>
@@ -4399,7 +4399,7 @@
         <v>ft601_data[31]</v>
       </c>
       <c r="J69" s="3" t="str">
-        <f>IF(I69&lt;&gt;"","IO_LOC """&amp;I69&amp;""" "&amp;D69&amp;";", "")</f>
+        <f t="shared" ref="J69:J100" si="2">IF(I69&lt;&gt;"","IO_LOC """&amp;I69&amp;""" "&amp;D69&amp;";", "")</f>
         <v>IO_LOC "ft601_data[31]" J2;</v>
       </c>
     </row>
@@ -4414,7 +4414,7 @@
         <v>40</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>49</v>
@@ -4431,7 +4431,7 @@
         <v>ft601_data[4]</v>
       </c>
       <c r="J70" s="3" t="str">
-        <f>IF(I70&lt;&gt;"","IO_LOC """&amp;I70&amp;""" "&amp;D70&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_data[4]" L8;</v>
       </c>
     </row>
@@ -4446,7 +4446,7 @@
         <v>38</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>50</v>
@@ -4463,7 +4463,7 @@
         <v>ft601_data[5]</v>
       </c>
       <c r="J71" s="3" t="str">
-        <f>IF(I71&lt;&gt;"","IO_LOC """&amp;I71&amp;""" "&amp;D71&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_data[5]" L7;</v>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
         <v>36</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>51</v>
@@ -4495,7 +4495,7 @@
         <v>ft601_data[6]</v>
       </c>
       <c r="J72" s="3" t="str">
-        <f>IF(I72&lt;&gt;"","IO_LOC """&amp;I72&amp;""" "&amp;D72&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_data[6]" J7;</v>
       </c>
     </row>
@@ -4510,10 +4510,10 @@
         <v>34</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="F73" s="4">
         <v>7</v>
@@ -4527,7 +4527,7 @@
         <v>ft601_data[7]</v>
       </c>
       <c r="J73" s="3" t="str">
-        <f>IF(I73&lt;&gt;"","IO_LOC """&amp;I73&amp;""" "&amp;D73&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_data[7]" K7;</v>
       </c>
     </row>
@@ -4542,7 +4542,7 @@
         <v>32</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>53</v>
@@ -4559,7 +4559,7 @@
         <v>ft601_data[8]</v>
       </c>
       <c r="J74" s="3" t="str">
-        <f>IF(I74&lt;&gt;"","IO_LOC """&amp;I74&amp;""" "&amp;D74&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_data[8]" K6;</v>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
         <v>30</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>54</v>
@@ -4591,7 +4591,7 @@
         <v>ft601_data[9]</v>
       </c>
       <c r="J75" s="3" t="str">
-        <f>IF(I75&lt;&gt;"","IO_LOC """&amp;I75&amp;""" "&amp;D75&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_data[9]" L6;</v>
       </c>
     </row>
@@ -4606,10 +4606,10 @@
         <v>34</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="F76" s="4">
         <v>3</v>
@@ -4625,7 +4625,7 @@
         <v>ft601_gpio[0]</v>
       </c>
       <c r="J76" s="3" t="str">
-        <f>IF(I76&lt;&gt;"","IO_LOC """&amp;I76&amp;""" "&amp;D76&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_gpio[0]" H1;</v>
       </c>
     </row>
@@ -4640,10 +4640,10 @@
         <v>36</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="F77" s="4">
         <v>3</v>
@@ -4659,7 +4659,7 @@
         <v>ft601_gpio[1]</v>
       </c>
       <c r="J77" s="3" t="str">
-        <f>IF(I77&lt;&gt;"","IO_LOC """&amp;I77&amp;""" "&amp;D77&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_gpio[1]" H2;</v>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
         <v>ft601_oe_n</v>
       </c>
       <c r="J78" s="3" t="str">
-        <f>IF(I78&lt;&gt;"","IO_LOC """&amp;I78&amp;""" "&amp;D78&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_oe_n" L1;</v>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
         <v>ft601_rd_n</v>
       </c>
       <c r="J79" s="3" t="str">
-        <f>IF(I79&lt;&gt;"","IO_LOC """&amp;I79&amp;""" "&amp;D79&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_rd_n" K1;</v>
       </c>
     </row>
@@ -4738,10 +4738,10 @@
         <v>6</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F80" s="4">
         <v>2</v>
@@ -4755,7 +4755,7 @@
         <v>ft601_reset_n</v>
       </c>
       <c r="J80" s="3" t="str">
-        <f>IF(I80&lt;&gt;"","IO_LOC """&amp;I80&amp;""" "&amp;D80&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_reset_n" L2;</v>
       </c>
     </row>
@@ -4787,7 +4787,7 @@
         <v>ft601_rxf_n</v>
       </c>
       <c r="J81" s="3" t="str">
-        <f>IF(I81&lt;&gt;"","IO_LOC """&amp;I81&amp;""" "&amp;D81&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_rxf_n" K4;</v>
       </c>
     </row>
@@ -4819,7 +4819,7 @@
         <v>ft601_siwu_n</v>
       </c>
       <c r="J82" s="3" t="str">
-        <f>IF(I82&lt;&gt;"","IO_LOC """&amp;I82&amp;""" "&amp;D82&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_siwu_n" J4;</v>
       </c>
     </row>
@@ -4834,16 +4834,16 @@
         <v>18</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F83" s="4">
         <v>2</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="H83" s="3">
         <v>1.8</v>
@@ -4853,7 +4853,7 @@
         <v>ft601_txe_n</v>
       </c>
       <c r="J83" s="3" t="str">
-        <f>IF(I83&lt;&gt;"","IO_LOC """&amp;I83&amp;""" "&amp;D83&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_txe_n" G2;</v>
       </c>
     </row>
@@ -4868,10 +4868,10 @@
         <v>32</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F84" s="4">
         <v>3</v>
@@ -4887,7 +4887,7 @@
         <v>ft601_wakeup</v>
       </c>
       <c r="J84" s="3" t="str">
-        <f>IF(I84&lt;&gt;"","IO_LOC """&amp;I84&amp;""" "&amp;D84&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_wakeup" H4;</v>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
         <v>ft601_wr_n</v>
       </c>
       <c r="J85" s="3" t="str">
-        <f>IF(I85&lt;&gt;"","IO_LOC """&amp;I85&amp;""" "&amp;D85&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "ft601_wr_n" K2;</v>
       </c>
     </row>
@@ -4930,10 +4930,10 @@
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
       <c r="D86" s="4" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="F86" s="4">
         <v>5</v>
@@ -4943,10 +4943,10 @@
         <v>3.3</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="J86" s="3" t="str">
-        <f>IF(I86&lt;&gt;"","IO_LOC """&amp;I86&amp;""" "&amp;D86&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "in_clk50" E2;</v>
       </c>
     </row>
@@ -4961,10 +4961,10 @@
         <v>21</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F87" s="4">
         <v>10</v>
@@ -4974,10 +4974,10 @@
         <v>3.3</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="J87" s="3" t="str">
-        <f>IF(I87&lt;&gt;"","IO_LOC """&amp;I87&amp;""" "&amp;D87&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "JTAG" C1;</v>
       </c>
     </row>
@@ -4992,10 +4992,10 @@
         <v>23</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F88" s="4">
         <v>10</v>
@@ -5005,10 +5005,10 @@
         <v>3.3</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="J88" s="3" t="str">
-        <f>IF(I88&lt;&gt;"","IO_LOC """&amp;I88&amp;""" "&amp;D88&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "JTAG" B1;</v>
       </c>
     </row>
@@ -5023,10 +5023,10 @@
         <v>25</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="F89" s="4">
         <v>10</v>
@@ -5036,10 +5036,10 @@
         <v>3.3</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="J89" s="3" t="str">
-        <f>IF(I89&lt;&gt;"","IO_LOC """&amp;I89&amp;""" "&amp;D89&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "JTAG" A2;</v>
       </c>
     </row>
@@ -5054,10 +5054,10 @@
         <v>27</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="F90" s="4">
         <v>10</v>
@@ -5067,10 +5067,10 @@
         <v>3.3</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="J90" s="3" t="str">
-        <f>IF(I90&lt;&gt;"","IO_LOC """&amp;I90&amp;""" "&amp;D90&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "JTAG" A3;</v>
       </c>
     </row>
@@ -5085,7 +5085,7 @@
         <v>52</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E91" s="4" t="s">
         <v>178</v>
@@ -5096,10 +5096,10 @@
       <c r="G91" s="4"/>
       <c r="H91" s="3"/>
       <c r="I91" s="3" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="J91" s="3" t="str">
-        <f>IF(I91&lt;&gt;"","IO_LOC """&amp;I91&amp;""" "&amp;D91&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "led[0]" E11;</v>
       </c>
     </row>
@@ -5114,10 +5114,10 @@
         <v>54</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>179</v>
+        <v>351</v>
       </c>
       <c r="F92" s="4">
         <v>6</v>
@@ -5125,10 +5125,10 @@
       <c r="G92" s="4"/>
       <c r="H92" s="3"/>
       <c r="I92" s="3" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="J92" s="3" t="str">
-        <f>IF(I92&lt;&gt;"","IO_LOC """&amp;I92&amp;""" "&amp;D92&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "led[1]" E10;</v>
       </c>
     </row>
@@ -5143,10 +5143,10 @@
         <v>56</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>180</v>
+        <v>352</v>
       </c>
       <c r="F93" s="4">
         <v>6</v>
@@ -5154,10 +5154,10 @@
       <c r="G93" s="4"/>
       <c r="H93" s="3"/>
       <c r="I93" s="3" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="J93" s="3" t="str">
-        <f>IF(I93&lt;&gt;"","IO_LOC """&amp;I93&amp;""" "&amp;D93&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "led[2]" A11;</v>
       </c>
     </row>
@@ -5172,10 +5172,10 @@
         <v>58</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>181</v>
+        <v>353</v>
       </c>
       <c r="F94" s="4">
         <v>6</v>
@@ -5183,10 +5183,10 @@
       <c r="G94" s="4"/>
       <c r="H94" s="3"/>
       <c r="I94" s="3" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="J94" s="3" t="str">
-        <f>IF(I94&lt;&gt;"","IO_LOC """&amp;I94&amp;""" "&amp;D94&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "led[3]" A10;</v>
       </c>
     </row>
@@ -5201,19 +5201,19 @@
         <v>45</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="F95" s="4"/>
       <c r="G95" s="4"/>
       <c r="H95" s="3"/>
       <c r="I95" s="3" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="J95" s="3" t="str">
-        <f>IF(I95&lt;&gt;"","IO_LOC """&amp;I95&amp;""" "&amp;D95&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "mipi_ck_n" B7;</v>
       </c>
     </row>
@@ -5228,19 +5228,19 @@
         <v>43</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F96" s="4"/>
       <c r="G96" s="4"/>
       <c r="H96" s="3"/>
       <c r="I96" s="3" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="J96" s="3" t="str">
-        <f>IF(I96&lt;&gt;"","IO_LOC """&amp;I96&amp;""" "&amp;D96&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "mipi_ck_p" A7;</v>
       </c>
     </row>
@@ -5255,19 +5255,19 @@
         <v>51</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="F97" s="4"/>
       <c r="G97" s="4"/>
       <c r="H97" s="3"/>
       <c r="I97" s="3" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="J97" s="3" t="str">
-        <f>IF(I97&lt;&gt;"","IO_LOC """&amp;I97&amp;""" "&amp;D97&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "mipi_d_n[1]" B8;</v>
       </c>
     </row>
@@ -5282,19 +5282,19 @@
         <v>57</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F98" s="4"/>
       <c r="G98" s="4"/>
       <c r="H98" s="3"/>
       <c r="I98" s="3" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="J98" s="3" t="str">
-        <f>IF(I98&lt;&gt;"","IO_LOC """&amp;I98&amp;""" "&amp;D98&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "mipi_d_n[1]" B9;</v>
       </c>
     </row>
@@ -5309,19 +5309,19 @@
         <v>39</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="F99" s="4"/>
       <c r="G99" s="4"/>
       <c r="H99" s="3"/>
       <c r="I99" s="3" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="J99" s="3" t="str">
-        <f>IF(I99&lt;&gt;"","IO_LOC """&amp;I99&amp;""" "&amp;D99&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "mipi_d_n[2]" B6;</v>
       </c>
     </row>
@@ -5336,19 +5336,19 @@
         <v>33</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F100" s="4"/>
       <c r="G100" s="4"/>
       <c r="H100" s="3"/>
       <c r="I100" s="3" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="J100" s="3" t="str">
-        <f>IF(I100&lt;&gt;"","IO_LOC """&amp;I100&amp;""" "&amp;D100&amp;";", "")</f>
+        <f t="shared" si="2"/>
         <v>IO_LOC "mipi_d_n[3]" B5;</v>
       </c>
     </row>
@@ -5363,19 +5363,19 @@
         <v>49</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="F101" s="4"/>
       <c r="G101" s="4"/>
       <c r="H101" s="3"/>
       <c r="I101" s="3" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="J101" s="3" t="str">
-        <f>IF(I101&lt;&gt;"","IO_LOC """&amp;I101&amp;""" "&amp;D101&amp;";", "")</f>
+        <f t="shared" ref="J101:J132" si="3">IF(I101&lt;&gt;"","IO_LOC """&amp;I101&amp;""" "&amp;D101&amp;";", "")</f>
         <v>IO_LOC "mipi_d_p[1]" A8;</v>
       </c>
     </row>
@@ -5390,19 +5390,19 @@
         <v>55</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F102" s="4"/>
       <c r="G102" s="4"/>
       <c r="H102" s="3"/>
       <c r="I102" s="3" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="J102" s="3" t="str">
-        <f>IF(I102&lt;&gt;"","IO_LOC """&amp;I102&amp;""" "&amp;D102&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_d_p[1]" A9;</v>
       </c>
     </row>
@@ -5417,19 +5417,19 @@
         <v>37</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="F103" s="4"/>
       <c r="G103" s="4"/>
       <c r="H103" s="3"/>
       <c r="I103" s="3" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="J103" s="3" t="str">
-        <f>IF(I103&lt;&gt;"","IO_LOC """&amp;I103&amp;""" "&amp;D103&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_d_p[2]" A6;</v>
       </c>
     </row>
@@ -5444,19 +5444,19 @@
         <v>31</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F104" s="4"/>
       <c r="G104" s="4"/>
       <c r="H104" s="3"/>
       <c r="I104" s="3" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="J104" s="3" t="str">
-        <f>IF(I104&lt;&gt;"","IO_LOC """&amp;I104&amp;""" "&amp;D104&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_d_p[3]" A5;</v>
       </c>
     </row>
@@ -5471,10 +5471,10 @@
         <v>11</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F105" s="4">
         <v>5</v>
@@ -5484,10 +5484,10 @@
         <v>3.3</v>
       </c>
       <c r="I105" s="3" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="J105" s="3" t="str">
-        <f>IF(I105&lt;&gt;"","IO_LOC """&amp;I105&amp;""" "&amp;D105&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_gpio[0]" A1;</v>
       </c>
     </row>
@@ -5502,10 +5502,10 @@
         <v>23</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F106" s="4">
         <v>4</v>
@@ -5515,10 +5515,10 @@
         <v>3.3</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="J106" s="3" t="str">
-        <f>IF(I106&lt;&gt;"","IO_LOC """&amp;I106&amp;""" "&amp;D106&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_gpio[1]" E3;</v>
       </c>
     </row>
@@ -5533,7 +5533,7 @@
         <v>43</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E107" s="4" t="s">
         <v>76</v>
@@ -5546,10 +5546,10 @@
         <v>1.8</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="J107" s="3" t="str">
-        <f>IF(I107&lt;&gt;"","IO_LOC """&amp;I107&amp;""" "&amp;D107&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_pwr_en" G10;</v>
       </c>
     </row>
@@ -5564,7 +5564,7 @@
         <v>47</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E108" s="4" t="s">
         <v>77</v>
@@ -5577,10 +5577,10 @@
         <v>1.8</v>
       </c>
       <c r="I108" s="3" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="J108" s="3" t="str">
-        <f>IF(I108&lt;&gt;"","IO_LOC """&amp;I108&amp;""" "&amp;D108&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_scl" D11;</v>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
         <v>49</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E109" s="4" t="s">
         <v>37</v>
@@ -5608,10 +5608,10 @@
         <v>1.8</v>
       </c>
       <c r="I109" s="3" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="J109" s="3" t="str">
-        <f>IF(I109&lt;&gt;"","IO_LOC """&amp;I109&amp;""" "&amp;D109&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "mipi_sda" D10;</v>
       </c>
     </row>
@@ -5626,10 +5626,10 @@
         <v>7</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F110" s="4">
         <v>5</v>
@@ -5641,10 +5641,10 @@
         <v>3.3</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="J110" s="3" t="str">
-        <f>IF(I110&lt;&gt;"","IO_LOC """&amp;I110&amp;""" "&amp;D110&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[0]" F2;</v>
       </c>
     </row>
@@ -5659,10 +5659,10 @@
         <v>9</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F111" s="4">
         <v>5</v>
@@ -5674,10 +5674,10 @@
         <v>3.3</v>
       </c>
       <c r="I111" s="3" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="J111" s="3" t="str">
-        <f>IF(I111&lt;&gt;"","IO_LOC """&amp;I111&amp;""" "&amp;D111&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[1]" F1;</v>
       </c>
     </row>
@@ -5692,10 +5692,10 @@
         <v>3</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="F112" s="4">
         <v>5</v>
@@ -5705,10 +5705,10 @@
         <v>3.3</v>
       </c>
       <c r="I112" s="3" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="J112" s="3" t="str">
-        <f>IF(I112&lt;&gt;"","IO_LOC """&amp;I112&amp;""" "&amp;D112&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[2]" B2;</v>
       </c>
     </row>
@@ -5723,10 +5723,10 @@
         <v>5</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="F113" s="4">
         <v>5</v>
@@ -5736,10 +5736,10 @@
         <v>3.3</v>
       </c>
       <c r="I113" s="3" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="J113" s="3" t="str">
-        <f>IF(I113&lt;&gt;"","IO_LOC """&amp;I113&amp;""" "&amp;D113&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[3]" C2;</v>
       </c>
     </row>
@@ -5754,10 +5754,10 @@
         <v>15</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="F114" s="4">
         <v>5</v>
@@ -5769,10 +5769,10 @@
         <v>3.3</v>
       </c>
       <c r="I114" s="3" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="J114" s="3" t="str">
-        <f>IF(I114&lt;&gt;"","IO_LOC """&amp;I114&amp;""" "&amp;D114&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[4]" E1;</v>
       </c>
     </row>
@@ -5787,10 +5787,10 @@
         <v>17</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="F115" s="4">
         <v>5</v>
@@ -5800,10 +5800,10 @@
         <v>3.3</v>
       </c>
       <c r="I115" s="3" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="J115" s="3" t="str">
-        <f>IF(I115&lt;&gt;"","IO_LOC """&amp;I115&amp;""" "&amp;D115&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[5]" D1;</v>
       </c>
     </row>
@@ -5818,10 +5818,10 @@
         <v>19</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="F116" s="4">
         <v>4</v>
@@ -5831,10 +5831,10 @@
         <v>3.3</v>
       </c>
       <c r="I116" s="3" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="J116" s="3" t="str">
-        <f>IF(I116&lt;&gt;"","IO_LOC """&amp;I116&amp;""" "&amp;D116&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[6]" B3;</v>
       </c>
     </row>
@@ -5849,10 +5849,10 @@
         <v>21</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F117" s="4">
         <v>4</v>
@@ -5862,10 +5862,10 @@
         <v>3.3</v>
       </c>
       <c r="I117" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="J117" s="3" t="str">
-        <f>IF(I117&lt;&gt;"","IO_LOC """&amp;I117&amp;""" "&amp;D117&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "pmod[7]" C3;</v>
       </c>
     </row>
@@ -5880,10 +5880,10 @@
         <v>55</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F118" s="4">
         <v>6</v>
@@ -5893,10 +5893,10 @@
         <v>1.8</v>
       </c>
       <c r="I118" s="3" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="J118" s="3" t="str">
-        <f>IF(I118&lt;&gt;"","IO_LOC """&amp;I118&amp;""" "&amp;D118&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "push_sw[0]" B11;</v>
       </c>
     </row>
@@ -5911,10 +5911,10 @@
         <v>57</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F119" s="4">
         <v>6</v>
@@ -5924,10 +5924,10 @@
         <v>1.8</v>
       </c>
       <c r="I119" s="3" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="J119" s="3" t="str">
-        <f>IF(I119&lt;&gt;"","IO_LOC """&amp;I119&amp;""" "&amp;D119&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "push_sw[1]" B10;</v>
       </c>
     </row>
@@ -5942,10 +5942,10 @@
         <v>17</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="F120" s="4">
         <v>4</v>
@@ -5955,10 +5955,10 @@
         <v>3.3</v>
       </c>
       <c r="I120" s="3" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="J120" s="3" t="str">
-        <f>IF(I120&lt;&gt;"","IO_LOC """&amp;I120&amp;""" "&amp;D120&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "test[0]" E8;</v>
       </c>
     </row>
@@ -5973,10 +5973,10 @@
         <v>25</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="F121" s="4">
         <v>4</v>
@@ -5986,10 +5986,10 @@
         <v>3.3</v>
       </c>
       <c r="I121" s="3" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="J121" s="3" t="str">
-        <f>IF(I121&lt;&gt;"","IO_LOC """&amp;I121&amp;""" "&amp;D121&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v>IO_LOC "test[1]" D7;</v>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       <c r="H122" s="3"/>
       <c r="I122" s="3"/>
       <c r="J122" s="3" t="str">
-        <f>IF(I122&lt;&gt;"","IO_LOC """&amp;I122&amp;""" "&amp;D122&amp;";", "")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update active layer in PCB design to layer 6
</commit_message>
<xml_diff>
--- a/doc/pin_assign.xlsx
+++ b/doc/pin_assign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e643ea309c96c6f6/Documents/Development/kicad/rtcl-tp25k-usb3/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="634" documentId="13_ncr:1_{704F26EB-9FE7-473F-96D3-0C973174CAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BF1F114-A25A-48FC-B7AC-6EF32D47EAE1}"/>
+  <xr:revisionPtr revIDLastSave="642" documentId="13_ncr:1_{704F26EB-9FE7-473F-96D3-0C973174CAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2714D9EA-FBB5-4FB9-A201-FEEFD2A9F50E}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="57840" yWindow="13710" windowWidth="26130" windowHeight="17970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6610" yWindow="3200" windowWidth="27280" windowHeight="15580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1170,107 +1170,110 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>push_sw[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>push_sw[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>dip_sw[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>dip_sw[1]</t>
+  </si>
+  <si>
+    <t>test[0]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>test[1]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A5</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B5</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A6</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B6</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A7</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B7</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A8</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B8</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A9</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B9</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B11_IOL12A</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>B10_IOL12B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C11_IOL5A</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>C10_IOL5B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>E10_IOL3B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A11_IOL14A</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A10_IOL14B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>led[1]</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>led[2]</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>led[3]</t>
-  </si>
-  <si>
-    <t>push_sw[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>push_sw[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>dip_sw[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>dip_sw[1]</t>
-  </si>
-  <si>
-    <t>test[0]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>test[1]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A5</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B5</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A6</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B6</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A7</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B7</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A8</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B8</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A9</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B9</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>No.</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B11_IOL12A</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>B10_IOL12B</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C11_IOL5A</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>C10_IOL5B</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>E10_IOL3B</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A11_IOL14A</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>A10_IOL14B</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2370,7 +2373,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18.5" thickBot="1">
       <c r="A1" s="7" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>173</v>
@@ -2402,47 +2405,53 @@
     </row>
     <row r="2" spans="1:10" ht="18.5" thickTop="1">
       <c r="A2" s="5">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>174</v>
+        <v>82</v>
       </c>
       <c r="C2" s="6">
-        <v>2</v>
-      </c>
-      <c r="D2" s="6"/>
+        <v>13</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>267</v>
+      </c>
       <c r="E2" s="6" t="s">
-        <v>176</v>
+        <v>310</v>
       </c>
       <c r="F2" s="6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G2" s="6"/>
-      <c r="H2" s="5"/>
+      <c r="H2" s="5">
+        <v>3.3</v>
+      </c>
       <c r="I2" s="5" t="str">
         <f>_xlfn.XLOOKUP(D2, Sheet1!B$2:B$48, Sheet1!A$2:A$48, "")</f>
         <v/>
       </c>
       <c r="J2" s="5" t="str">
-        <f t="shared" ref="J2:J35" si="0">IF(I2&lt;&gt;"","IO_LOC """&amp;I2&amp;""" "&amp;D2&amp;";", "")</f>
+        <f>IF(I2&lt;&gt;"","IO_LOC """&amp;I2&amp;""" "&amp;D2&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C3" s="4">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="F3" s="4"/>
+        <v>176</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3" t="str">
@@ -2450,19 +2459,19 @@
         <v/>
       </c>
       <c r="J3" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I3&lt;&gt;"","IO_LOC """&amp;I3&amp;""" "&amp;D3&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C4" s="4">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
@@ -2476,23 +2485,23 @@
         <v/>
       </c>
       <c r="J4" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I4&lt;&gt;"","IO_LOC """&amp;I4&amp;""" "&amp;D4&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C5" s="4">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -2502,19 +2511,19 @@
         <v/>
       </c>
       <c r="J5" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I5&lt;&gt;"","IO_LOC """&amp;I5&amp;""" "&amp;D5&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="3">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C6" s="4">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4" t="s">
@@ -2528,19 +2537,19 @@
         <v/>
       </c>
       <c r="J6" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I6&lt;&gt;"","IO_LOC """&amp;I6&amp;""" "&amp;D6&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="3">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C7" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4" t="s">
@@ -2554,27 +2563,25 @@
         <v/>
       </c>
       <c r="J7" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I7&lt;&gt;"","IO_LOC """&amp;I7&amp;""" "&amp;D7&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="3">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C8" s="4">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F8" s="4">
-        <v>0</v>
-      </c>
+      <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3" t="str">
@@ -2582,25 +2589,27 @@
         <v/>
       </c>
       <c r="J8" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I8&lt;&gt;"","IO_LOC """&amp;I8&amp;""" "&amp;D8&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="3">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C9" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F9" s="4"/>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3" t="str">
@@ -2608,19 +2617,19 @@
         <v/>
       </c>
       <c r="J9" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I9&lt;&gt;"","IO_LOC """&amp;I9&amp;""" "&amp;D9&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="3">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C10" s="4">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
@@ -2634,23 +2643,23 @@
         <v/>
       </c>
       <c r="J10" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I10&lt;&gt;"","IO_LOC """&amp;I10&amp;""" "&amp;D10&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="3">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C11" s="4">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -2660,19 +2669,19 @@
         <v/>
       </c>
       <c r="J11" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I11&lt;&gt;"","IO_LOC """&amp;I11&amp;""" "&amp;D11&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C12" s="4">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
@@ -2686,23 +2695,23 @@
         <v/>
       </c>
       <c r="J12" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I12&lt;&gt;"","IO_LOC """&amp;I12&amp;""" "&amp;D12&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="3">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C13" s="4">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -2712,19 +2721,19 @@
         <v/>
       </c>
       <c r="J13" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I13&lt;&gt;"","IO_LOC """&amp;I13&amp;""" "&amp;D13&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="3">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C14" s="4">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
@@ -2738,23 +2747,23 @@
         <v/>
       </c>
       <c r="J14" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I14&lt;&gt;"","IO_LOC """&amp;I14&amp;""" "&amp;D14&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="3">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>82</v>
+        <v>174</v>
       </c>
       <c r="C15" s="4">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>233</v>
+        <v>176</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -2764,19 +2773,19 @@
         <v/>
       </c>
       <c r="J15" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I15&lt;&gt;"","IO_LOC """&amp;I15&amp;""" "&amp;D15&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="3">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C16" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
@@ -2790,23 +2799,23 @@
         <v/>
       </c>
       <c r="J16" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I16&lt;&gt;"","IO_LOC """&amp;I16&amp;""" "&amp;D16&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C17" s="4">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -2816,19 +2825,19 @@
         <v/>
       </c>
       <c r="J17" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I17&lt;&gt;"","IO_LOC """&amp;I17&amp;""" "&amp;D17&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C18" s="4">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
@@ -2842,23 +2851,23 @@
         <v/>
       </c>
       <c r="J18" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I18&lt;&gt;"","IO_LOC """&amp;I18&amp;""" "&amp;D18&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C19" s="4">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -2868,19 +2877,19 @@
         <v/>
       </c>
       <c r="J19" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I19&lt;&gt;"","IO_LOC """&amp;I19&amp;""" "&amp;D19&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="3">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C20" s="4">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
@@ -2894,23 +2903,23 @@
         <v/>
       </c>
       <c r="J20" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I20&lt;&gt;"","IO_LOC """&amp;I20&amp;""" "&amp;D20&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C21" s="4">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -2920,19 +2929,19 @@
         <v/>
       </c>
       <c r="J21" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I21&lt;&gt;"","IO_LOC """&amp;I21&amp;""" "&amp;D21&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="3">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C22" s="4">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
@@ -2946,19 +2955,19 @@
         <v/>
       </c>
       <c r="J22" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I22&lt;&gt;"","IO_LOC """&amp;I22&amp;""" "&amp;D22&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="3">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C23" s="4">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
@@ -2972,23 +2981,23 @@
         <v/>
       </c>
       <c r="J23" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I23&lt;&gt;"","IO_LOC """&amp;I23&amp;""" "&amp;D23&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="3">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C24" s="4">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -2998,19 +3007,19 @@
         <v/>
       </c>
       <c r="J24" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I24&lt;&gt;"","IO_LOC """&amp;I24&amp;""" "&amp;D24&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="3">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C25" s="4">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
@@ -3024,19 +3033,19 @@
         <v/>
       </c>
       <c r="J25" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I25&lt;&gt;"","IO_LOC """&amp;I25&amp;""" "&amp;D25&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="3">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C26" s="4">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
@@ -3050,19 +3059,19 @@
         <v/>
       </c>
       <c r="J26" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I26&lt;&gt;"","IO_LOC """&amp;I26&amp;""" "&amp;D26&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="3">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C27" s="4">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
@@ -3076,19 +3085,19 @@
         <v/>
       </c>
       <c r="J27" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I27&lt;&gt;"","IO_LOC """&amp;I27&amp;""" "&amp;D27&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="3">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C28" s="4">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
@@ -3102,23 +3111,23 @@
         <v/>
       </c>
       <c r="J28" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I28&lt;&gt;"","IO_LOC """&amp;I28&amp;""" "&amp;D28&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="3">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C29" s="4">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4" t="s">
-        <v>176</v>
+        <v>246</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -3128,39 +3137,33 @@
         <v/>
       </c>
       <c r="J29" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I29&lt;&gt;"","IO_LOC """&amp;I29&amp;""" "&amp;D29&amp;";", "")</f>
         <v/>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="3">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C30" s="4">
-        <v>13</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>267</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="F30" s="4">
-        <v>5</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="F30" s="4"/>
       <c r="G30" s="4"/>
-      <c r="H30" s="3">
-        <v>3.3</v>
-      </c>
+      <c r="H30" s="3"/>
       <c r="I30" s="3" t="str">
         <f>_xlfn.XLOOKUP(D30, Sheet1!B$2:B$48, Sheet1!A$2:A$48, "")</f>
         <v/>
       </c>
       <c r="J30" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I30&lt;&gt;"","IO_LOC """&amp;I30&amp;""" "&amp;D30&amp;";", "")</f>
         <v/>
       </c>
     </row>
@@ -3186,7 +3189,7 @@
         <v/>
       </c>
       <c r="J31" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I31&lt;&gt;"","IO_LOC """&amp;I31&amp;""" "&amp;D31&amp;";", "")</f>
         <v/>
       </c>
     </row>
@@ -3212,7 +3215,7 @@
         <v/>
       </c>
       <c r="J32" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I32&lt;&gt;"","IO_LOC """&amp;I32&amp;""" "&amp;D32&amp;";", "")</f>
         <v/>
       </c>
     </row>
@@ -3238,7 +3241,7 @@
         <v/>
       </c>
       <c r="J33" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I33&lt;&gt;"","IO_LOC """&amp;I33&amp;""" "&amp;D33&amp;";", "")</f>
         <v/>
       </c>
     </row>
@@ -3264,7 +3267,7 @@
         <v/>
       </c>
       <c r="J34" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I34&lt;&gt;"","IO_LOC """&amp;I34&amp;""" "&amp;D34&amp;";", "")</f>
         <v/>
       </c>
     </row>
@@ -3290,7 +3293,7 @@
         <v/>
       </c>
       <c r="J35" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(I35&lt;&gt;"","IO_LOC """&amp;I35&amp;""" "&amp;D35&amp;";", "")</f>
         <v/>
       </c>
     </row>
@@ -3331,7 +3334,7 @@
         <v>223</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F37" s="4">
         <v>6</v>
@@ -3341,10 +3344,10 @@
         <v>1.8</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="J37" s="3" t="str">
-        <f t="shared" ref="J37:J68" si="1">IF(I37&lt;&gt;"","IO_LOC """&amp;I37&amp;""" "&amp;D37&amp;";", "")</f>
+        <f>IF(I37&lt;&gt;"","IO_LOC """&amp;I37&amp;""" "&amp;D37&amp;";", "")</f>
         <v>IO_LOC "dip_sw[0]" C11;</v>
       </c>
     </row>
@@ -3362,7 +3365,7 @@
         <v>224</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F38" s="4">
         <v>6</v>
@@ -3372,10 +3375,10 @@
         <v>1.8</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="J38" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I38&lt;&gt;"","IO_LOC """&amp;I38&amp;""" "&amp;D38&amp;";", "")</f>
         <v>IO_LOC "dip_sw[1]" C10;</v>
       </c>
     </row>
@@ -3409,7 +3412,7 @@
         <v>ft601_be[0]</v>
       </c>
       <c r="J39" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I39&lt;&gt;"","IO_LOC """&amp;I39&amp;""" "&amp;D39&amp;";", "")</f>
         <v>IO_LOC "ft601_be[0]" J1;</v>
       </c>
     </row>
@@ -3443,7 +3446,7 @@
         <v>ft601_be[1]</v>
       </c>
       <c r="J40" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I40&lt;&gt;"","IO_LOC """&amp;I40&amp;""" "&amp;D40&amp;";", "")</f>
         <v>IO_LOC "ft601_be[1]" L3;</v>
       </c>
     </row>
@@ -3477,7 +3480,7 @@
         <v>ft601_be[2]</v>
       </c>
       <c r="J41" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I41&lt;&gt;"","IO_LOC """&amp;I41&amp;""" "&amp;D41&amp;";", "")</f>
         <v>IO_LOC "ft601_be[2]" L4;</v>
       </c>
     </row>
@@ -3509,7 +3512,7 @@
         <v>ft601_be[3]</v>
       </c>
       <c r="J42" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I42&lt;&gt;"","IO_LOC """&amp;I42&amp;""" "&amp;D42&amp;";", "")</f>
         <v>IO_LOC "ft601_be[3]" G1;</v>
       </c>
     </row>
@@ -3543,7 +3546,7 @@
         <v>ft601_clk</v>
       </c>
       <c r="J43" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I43&lt;&gt;"","IO_LOC """&amp;I43&amp;""" "&amp;D43&amp;";", "")</f>
         <v>IO_LOC "ft601_clk" K5;</v>
       </c>
     </row>
@@ -3575,7 +3578,7 @@
         <v>ft601_data[0]</v>
       </c>
       <c r="J44" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I44&lt;&gt;"","IO_LOC """&amp;I44&amp;""" "&amp;D44&amp;";", "")</f>
         <v>IO_LOC "ft601_data[0]" L11;</v>
       </c>
     </row>
@@ -3607,7 +3610,7 @@
         <v>ft601_data[1]</v>
       </c>
       <c r="J45" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I45&lt;&gt;"","IO_LOC """&amp;I45&amp;""" "&amp;D45&amp;";", "")</f>
         <v>IO_LOC "ft601_data[1]" K11;</v>
       </c>
     </row>
@@ -3639,7 +3642,7 @@
         <v>ft601_data[10]</v>
       </c>
       <c r="J46" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I46&lt;&gt;"","IO_LOC """&amp;I46&amp;""" "&amp;D46&amp;";", "")</f>
         <v>IO_LOC "ft601_data[10]" G5;</v>
       </c>
     </row>
@@ -3671,7 +3674,7 @@
         <v>ft601_data[11]</v>
       </c>
       <c r="J47" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I47&lt;&gt;"","IO_LOC """&amp;I47&amp;""" "&amp;D47&amp;";", "")</f>
         <v>IO_LOC "ft601_data[11]" F5;</v>
       </c>
     </row>
@@ -3703,7 +3706,7 @@
         <v>ft601_data[12]</v>
       </c>
       <c r="J48" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I48&lt;&gt;"","IO_LOC """&amp;I48&amp;""" "&amp;D48&amp;";", "")</f>
         <v>IO_LOC "ft601_data[12]" G8;</v>
       </c>
     </row>
@@ -3735,7 +3738,7 @@
         <v>ft601_data[13]</v>
       </c>
       <c r="J49" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I49&lt;&gt;"","IO_LOC """&amp;I49&amp;""" "&amp;D49&amp;";", "")</f>
         <v>IO_LOC "ft601_data[13]" G7;</v>
       </c>
     </row>
@@ -3767,7 +3770,7 @@
         <v>ft601_data[14]</v>
       </c>
       <c r="J50" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I50&lt;&gt;"","IO_LOC """&amp;I50&amp;""" "&amp;D50&amp;";", "")</f>
         <v>IO_LOC "ft601_data[14]" H7;</v>
       </c>
     </row>
@@ -3799,7 +3802,7 @@
         <v>ft601_data[15]</v>
       </c>
       <c r="J51" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I51&lt;&gt;"","IO_LOC """&amp;I51&amp;""" "&amp;D51&amp;";", "")</f>
         <v>IO_LOC "ft601_data[15]" H8;</v>
       </c>
     </row>
@@ -3833,7 +3836,7 @@
         <v>ft601_data[16]</v>
       </c>
       <c r="J52" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I52&lt;&gt;"","IO_LOC """&amp;I52&amp;""" "&amp;D52&amp;";", "")</f>
         <v>IO_LOC "ft601_data[16]" H5;</v>
       </c>
     </row>
@@ -3867,7 +3870,7 @@
         <v>ft601_data[17]</v>
       </c>
       <c r="J53" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I53&lt;&gt;"","IO_LOC """&amp;I53&amp;""" "&amp;D53&amp;";", "")</f>
         <v>IO_LOC "ft601_data[17]" J5;</v>
       </c>
     </row>
@@ -3901,7 +3904,7 @@
         <v>ft601_data[18]</v>
       </c>
       <c r="J54" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I54&lt;&gt;"","IO_LOC """&amp;I54&amp;""" "&amp;D54&amp;";", "")</f>
         <v>IO_LOC "ft601_data[18]" L5;</v>
       </c>
     </row>
@@ -3933,7 +3936,7 @@
         <v>ft601_data[19]</v>
       </c>
       <c r="J55" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I55&lt;&gt;"","IO_LOC """&amp;I55&amp;""" "&amp;D55&amp;";", "")</f>
         <v>IO_LOC "ft601_data[19]" L9;</v>
       </c>
     </row>
@@ -3965,7 +3968,7 @@
         <v>ft601_data[2]</v>
       </c>
       <c r="J56" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I56&lt;&gt;"","IO_LOC """&amp;I56&amp;""" "&amp;D56&amp;";", "")</f>
         <v>IO_LOC "ft601_data[2]" K10;</v>
       </c>
     </row>
@@ -3997,7 +4000,7 @@
         <v>ft601_data[20]</v>
       </c>
       <c r="J57" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I57&lt;&gt;"","IO_LOC """&amp;I57&amp;""" "&amp;D57&amp;";", "")</f>
         <v>IO_LOC "ft601_data[20]" K9;</v>
       </c>
     </row>
@@ -4031,7 +4034,7 @@
         <v>ft601_data[21]</v>
       </c>
       <c r="J58" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I58&lt;&gt;"","IO_LOC """&amp;I58&amp;""" "&amp;D58&amp;";", "")</f>
         <v>IO_LOC "ft601_data[21]" J8;</v>
       </c>
     </row>
@@ -4065,7 +4068,7 @@
         <v>ft601_data[22]</v>
       </c>
       <c r="J59" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I59&lt;&gt;"","IO_LOC """&amp;I59&amp;""" "&amp;D59&amp;";", "")</f>
         <v>IO_LOC "ft601_data[22]" K8;</v>
       </c>
     </row>
@@ -4099,7 +4102,7 @@
         <v>ft601_data[23]</v>
       </c>
       <c r="J60" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I60&lt;&gt;"","IO_LOC """&amp;I60&amp;""" "&amp;D60&amp;";", "")</f>
         <v>IO_LOC "ft601_data[23]" F7;</v>
       </c>
     </row>
@@ -4131,7 +4134,7 @@
         <v>ft601_data[24]</v>
       </c>
       <c r="J61" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I61&lt;&gt;"","IO_LOC """&amp;I61&amp;""" "&amp;D61&amp;";", "")</f>
         <v>IO_LOC "ft601_data[24]" F6;</v>
       </c>
     </row>
@@ -4165,7 +4168,7 @@
         <v>ft601_data[25]</v>
       </c>
       <c r="J62" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I62&lt;&gt;"","IO_LOC """&amp;I62&amp;""" "&amp;D62&amp;";", "")</f>
         <v>IO_LOC "ft601_data[25]" J11;</v>
       </c>
     </row>
@@ -4199,7 +4202,7 @@
         <v>ft601_data[26]</v>
       </c>
       <c r="J63" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I63&lt;&gt;"","IO_LOC """&amp;I63&amp;""" "&amp;D63&amp;";", "")</f>
         <v>IO_LOC "ft601_data[26]" J10;</v>
       </c>
     </row>
@@ -4233,7 +4236,7 @@
         <v>ft601_data[27]</v>
       </c>
       <c r="J64" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I64&lt;&gt;"","IO_LOC """&amp;I64&amp;""" "&amp;D64&amp;";", "")</f>
         <v>IO_LOC "ft601_data[27]" H11;</v>
       </c>
     </row>
@@ -4267,7 +4270,7 @@
         <v>ft601_data[28]</v>
       </c>
       <c r="J65" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I65&lt;&gt;"","IO_LOC """&amp;I65&amp;""" "&amp;D65&amp;";", "")</f>
         <v>IO_LOC "ft601_data[28]" H10;</v>
       </c>
     </row>
@@ -4299,7 +4302,7 @@
         <v>ft601_data[29]</v>
       </c>
       <c r="J66" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I66&lt;&gt;"","IO_LOC """&amp;I66&amp;""" "&amp;D66&amp;";", "")</f>
         <v>IO_LOC "ft601_data[29]" G11;</v>
       </c>
     </row>
@@ -4331,7 +4334,7 @@
         <v>ft601_data[3]</v>
       </c>
       <c r="J67" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I67&lt;&gt;"","IO_LOC """&amp;I67&amp;""" "&amp;D67&amp;";", "")</f>
         <v>IO_LOC "ft601_data[3]" L10;</v>
       </c>
     </row>
@@ -4365,7 +4368,7 @@
         <v>ft601_data[30]</v>
       </c>
       <c r="J68" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(I68&lt;&gt;"","IO_LOC """&amp;I68&amp;""" "&amp;D68&amp;";", "")</f>
         <v>IO_LOC "ft601_data[30]" G4;</v>
       </c>
     </row>
@@ -4399,7 +4402,7 @@
         <v>ft601_data[31]</v>
       </c>
       <c r="J69" s="3" t="str">
-        <f t="shared" ref="J69:J100" si="2">IF(I69&lt;&gt;"","IO_LOC """&amp;I69&amp;""" "&amp;D69&amp;";", "")</f>
+        <f>IF(I69&lt;&gt;"","IO_LOC """&amp;I69&amp;""" "&amp;D69&amp;";", "")</f>
         <v>IO_LOC "ft601_data[31]" J2;</v>
       </c>
     </row>
@@ -4431,7 +4434,7 @@
         <v>ft601_data[4]</v>
       </c>
       <c r="J70" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I70&lt;&gt;"","IO_LOC """&amp;I70&amp;""" "&amp;D70&amp;";", "")</f>
         <v>IO_LOC "ft601_data[4]" L8;</v>
       </c>
     </row>
@@ -4463,7 +4466,7 @@
         <v>ft601_data[5]</v>
       </c>
       <c r="J71" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I71&lt;&gt;"","IO_LOC """&amp;I71&amp;""" "&amp;D71&amp;";", "")</f>
         <v>IO_LOC "ft601_data[5]" L7;</v>
       </c>
     </row>
@@ -4495,7 +4498,7 @@
         <v>ft601_data[6]</v>
       </c>
       <c r="J72" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I72&lt;&gt;"","IO_LOC """&amp;I72&amp;""" "&amp;D72&amp;";", "")</f>
         <v>IO_LOC "ft601_data[6]" J7;</v>
       </c>
     </row>
@@ -4527,7 +4530,7 @@
         <v>ft601_data[7]</v>
       </c>
       <c r="J73" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I73&lt;&gt;"","IO_LOC """&amp;I73&amp;""" "&amp;D73&amp;";", "")</f>
         <v>IO_LOC "ft601_data[7]" K7;</v>
       </c>
     </row>
@@ -4559,7 +4562,7 @@
         <v>ft601_data[8]</v>
       </c>
       <c r="J74" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I74&lt;&gt;"","IO_LOC """&amp;I74&amp;""" "&amp;D74&amp;";", "")</f>
         <v>IO_LOC "ft601_data[8]" K6;</v>
       </c>
     </row>
@@ -4591,7 +4594,7 @@
         <v>ft601_data[9]</v>
       </c>
       <c r="J75" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I75&lt;&gt;"","IO_LOC """&amp;I75&amp;""" "&amp;D75&amp;";", "")</f>
         <v>IO_LOC "ft601_data[9]" L6;</v>
       </c>
     </row>
@@ -4625,7 +4628,7 @@
         <v>ft601_gpio[0]</v>
       </c>
       <c r="J76" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I76&lt;&gt;"","IO_LOC """&amp;I76&amp;""" "&amp;D76&amp;";", "")</f>
         <v>IO_LOC "ft601_gpio[0]" H1;</v>
       </c>
     </row>
@@ -4659,7 +4662,7 @@
         <v>ft601_gpio[1]</v>
       </c>
       <c r="J77" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I77&lt;&gt;"","IO_LOC """&amp;I77&amp;""" "&amp;D77&amp;";", "")</f>
         <v>IO_LOC "ft601_gpio[1]" H2;</v>
       </c>
     </row>
@@ -4691,7 +4694,7 @@
         <v>ft601_oe_n</v>
       </c>
       <c r="J78" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I78&lt;&gt;"","IO_LOC """&amp;I78&amp;""" "&amp;D78&amp;";", "")</f>
         <v>IO_LOC "ft601_oe_n" L1;</v>
       </c>
     </row>
@@ -4723,7 +4726,7 @@
         <v>ft601_rd_n</v>
       </c>
       <c r="J79" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I79&lt;&gt;"","IO_LOC """&amp;I79&amp;""" "&amp;D79&amp;";", "")</f>
         <v>IO_LOC "ft601_rd_n" K1;</v>
       </c>
     </row>
@@ -4755,7 +4758,7 @@
         <v>ft601_reset_n</v>
       </c>
       <c r="J80" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I80&lt;&gt;"","IO_LOC """&amp;I80&amp;""" "&amp;D80&amp;";", "")</f>
         <v>IO_LOC "ft601_reset_n" L2;</v>
       </c>
     </row>
@@ -4787,7 +4790,7 @@
         <v>ft601_rxf_n</v>
       </c>
       <c r="J81" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I81&lt;&gt;"","IO_LOC """&amp;I81&amp;""" "&amp;D81&amp;";", "")</f>
         <v>IO_LOC "ft601_rxf_n" K4;</v>
       </c>
     </row>
@@ -4819,7 +4822,7 @@
         <v>ft601_siwu_n</v>
       </c>
       <c r="J82" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I82&lt;&gt;"","IO_LOC """&amp;I82&amp;""" "&amp;D82&amp;";", "")</f>
         <v>IO_LOC "ft601_siwu_n" J4;</v>
       </c>
     </row>
@@ -4853,7 +4856,7 @@
         <v>ft601_txe_n</v>
       </c>
       <c r="J83" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I83&lt;&gt;"","IO_LOC """&amp;I83&amp;""" "&amp;D83&amp;";", "")</f>
         <v>IO_LOC "ft601_txe_n" G2;</v>
       </c>
     </row>
@@ -4887,7 +4890,7 @@
         <v>ft601_wakeup</v>
       </c>
       <c r="J84" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I84&lt;&gt;"","IO_LOC """&amp;I84&amp;""" "&amp;D84&amp;";", "")</f>
         <v>IO_LOC "ft601_wakeup" H4;</v>
       </c>
     </row>
@@ -4919,7 +4922,7 @@
         <v>ft601_wr_n</v>
       </c>
       <c r="J85" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I85&lt;&gt;"","IO_LOC """&amp;I85&amp;""" "&amp;D85&amp;";", "")</f>
         <v>IO_LOC "ft601_wr_n" K2;</v>
       </c>
     </row>
@@ -4946,25 +4949,25 @@
         <v>315</v>
       </c>
       <c r="J86" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I86&lt;&gt;"","IO_LOC """&amp;I86&amp;""" "&amp;D86&amp;";", "")</f>
         <v>IO_LOC "in_clk50" E2;</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="3">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C87" s="4">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F87" s="4">
         <v>10</v>
@@ -4977,25 +4980,25 @@
         <v>293</v>
       </c>
       <c r="J87" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "JTAG" C1;</v>
+        <f>IF(I87&lt;&gt;"","IO_LOC """&amp;I87&amp;""" "&amp;D87&amp;";", "")</f>
+        <v>IO_LOC "JTAG" A2;</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="3">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C88" s="4">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="F88" s="4">
         <v>10</v>
@@ -5008,25 +5011,25 @@
         <v>293</v>
       </c>
       <c r="J88" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "JTAG" B1;</v>
+        <f>IF(I88&lt;&gt;"","IO_LOC """&amp;I88&amp;""" "&amp;D88&amp;";", "")</f>
+        <v>IO_LOC "JTAG" A3;</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="3">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C89" s="4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F89" s="4">
         <v>10</v>
@@ -5039,25 +5042,25 @@
         <v>293</v>
       </c>
       <c r="J89" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "JTAG" A2;</v>
+        <f>IF(I89&lt;&gt;"","IO_LOC """&amp;I89&amp;""" "&amp;D89&amp;";", "")</f>
+        <v>IO_LOC "JTAG" B1;</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="3">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C90" s="4">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F90" s="4">
         <v>10</v>
@@ -5070,8 +5073,8 @@
         <v>293</v>
       </c>
       <c r="J90" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "JTAG" A3;</v>
+        <f>IF(I90&lt;&gt;"","IO_LOC """&amp;I90&amp;""" "&amp;D90&amp;";", "")</f>
+        <v>IO_LOC "JTAG" C1;</v>
       </c>
     </row>
     <row r="91" spans="1:10">
@@ -5096,11 +5099,11 @@
       <c r="G91" s="4"/>
       <c r="H91" s="3"/>
       <c r="I91" s="3" t="s">
-        <v>305</v>
+        <v>353</v>
       </c>
       <c r="J91" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "led[0]" E11;</v>
+        <f>IF(I91&lt;&gt;"","IO_LOC """&amp;I91&amp;""" "&amp;D91&amp;";", "")</f>
+        <v>IO_LOC "led[3]" E11;</v>
       </c>
     </row>
     <row r="92" spans="1:10">
@@ -5117,7 +5120,7 @@
         <v>194</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F92" s="4">
         <v>6</v>
@@ -5125,11 +5128,11 @@
       <c r="G92" s="4"/>
       <c r="H92" s="3"/>
       <c r="I92" s="3" t="s">
-        <v>327</v>
+        <v>352</v>
       </c>
       <c r="J92" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "led[1]" E10;</v>
+        <f>IF(I92&lt;&gt;"","IO_LOC """&amp;I92&amp;""" "&amp;D92&amp;";", "")</f>
+        <v>IO_LOC "led[2]" E10;</v>
       </c>
     </row>
     <row r="93" spans="1:10">
@@ -5146,7 +5149,7 @@
         <v>232</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F93" s="4">
         <v>6</v>
@@ -5154,11 +5157,11 @@
       <c r="G93" s="4"/>
       <c r="H93" s="3"/>
       <c r="I93" s="3" t="s">
-        <v>328</v>
+        <v>351</v>
       </c>
       <c r="J93" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "led[2]" A11;</v>
+        <f>IF(I93&lt;&gt;"","IO_LOC """&amp;I93&amp;""" "&amp;D93&amp;";", "")</f>
+        <v>IO_LOC "led[1]" A11;</v>
       </c>
     </row>
     <row r="94" spans="1:10">
@@ -5175,7 +5178,7 @@
         <v>195</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F94" s="4">
         <v>6</v>
@@ -5183,11 +5186,11 @@
       <c r="G94" s="4"/>
       <c r="H94" s="3"/>
       <c r="I94" s="3" t="s">
-        <v>329</v>
+        <v>305</v>
       </c>
       <c r="J94" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>IO_LOC "led[3]" A10;</v>
+        <f>IF(I94&lt;&gt;"","IO_LOC """&amp;I94&amp;""" "&amp;D94&amp;";", "")</f>
+        <v>IO_LOC "led[0]" A10;</v>
       </c>
     </row>
     <row r="95" spans="1:10">
@@ -5201,7 +5204,7 @@
         <v>45</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E95" s="4" t="s">
         <v>280</v>
@@ -5213,7 +5216,7 @@
         <v>295</v>
       </c>
       <c r="J95" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I95&lt;&gt;"","IO_LOC """&amp;I95&amp;""" "&amp;D95&amp;";", "")</f>
         <v>IO_LOC "mipi_ck_n" B7;</v>
       </c>
     </row>
@@ -5228,7 +5231,7 @@
         <v>43</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E96" s="4" t="s">
         <v>279</v>
@@ -5240,7 +5243,7 @@
         <v>294</v>
       </c>
       <c r="J96" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I96&lt;&gt;"","IO_LOC """&amp;I96&amp;""" "&amp;D96&amp;";", "")</f>
         <v>IO_LOC "mipi_ck_p" A7;</v>
       </c>
     </row>
@@ -5255,7 +5258,7 @@
         <v>51</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E97" s="4" t="s">
         <v>282</v>
@@ -5267,7 +5270,7 @@
         <v>301</v>
       </c>
       <c r="J97" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I97&lt;&gt;"","IO_LOC """&amp;I97&amp;""" "&amp;D97&amp;";", "")</f>
         <v>IO_LOC "mipi_d_n[1]" B8;</v>
       </c>
     </row>
@@ -5282,7 +5285,7 @@
         <v>57</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>284</v>
@@ -5294,7 +5297,7 @@
         <v>301</v>
       </c>
       <c r="J98" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I98&lt;&gt;"","IO_LOC """&amp;I98&amp;""" "&amp;D98&amp;";", "")</f>
         <v>IO_LOC "mipi_d_n[1]" B9;</v>
       </c>
     </row>
@@ -5309,7 +5312,7 @@
         <v>39</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E99" s="4" t="s">
         <v>278</v>
@@ -5321,7 +5324,7 @@
         <v>299</v>
       </c>
       <c r="J99" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I99&lt;&gt;"","IO_LOC """&amp;I99&amp;""" "&amp;D99&amp;";", "")</f>
         <v>IO_LOC "mipi_d_n[2]" B6;</v>
       </c>
     </row>
@@ -5336,7 +5339,7 @@
         <v>33</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E100" s="4" t="s">
         <v>276</v>
@@ -5348,7 +5351,7 @@
         <v>297</v>
       </c>
       <c r="J100" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(I100&lt;&gt;"","IO_LOC """&amp;I100&amp;""" "&amp;D100&amp;";", "")</f>
         <v>IO_LOC "mipi_d_n[3]" B5;</v>
       </c>
     </row>
@@ -5363,7 +5366,7 @@
         <v>49</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="E101" s="4" t="s">
         <v>281</v>
@@ -5375,7 +5378,7 @@
         <v>300</v>
       </c>
       <c r="J101" s="3" t="str">
-        <f t="shared" ref="J101:J132" si="3">IF(I101&lt;&gt;"","IO_LOC """&amp;I101&amp;""" "&amp;D101&amp;";", "")</f>
+        <f>IF(I101&lt;&gt;"","IO_LOC """&amp;I101&amp;""" "&amp;D101&amp;";", "")</f>
         <v>IO_LOC "mipi_d_p[1]" A8;</v>
       </c>
     </row>
@@ -5390,7 +5393,7 @@
         <v>55</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="E102" s="4" t="s">
         <v>283</v>
@@ -5402,7 +5405,7 @@
         <v>300</v>
       </c>
       <c r="J102" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I102&lt;&gt;"","IO_LOC """&amp;I102&amp;""" "&amp;D102&amp;";", "")</f>
         <v>IO_LOC "mipi_d_p[1]" A9;</v>
       </c>
     </row>
@@ -5417,7 +5420,7 @@
         <v>37</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E103" s="4" t="s">
         <v>277</v>
@@ -5429,7 +5432,7 @@
         <v>298</v>
       </c>
       <c r="J103" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I103&lt;&gt;"","IO_LOC """&amp;I103&amp;""" "&amp;D103&amp;";", "")</f>
         <v>IO_LOC "mipi_d_p[2]" A6;</v>
       </c>
     </row>
@@ -5444,7 +5447,7 @@
         <v>31</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E104" s="4" t="s">
         <v>275</v>
@@ -5456,7 +5459,7 @@
         <v>296</v>
       </c>
       <c r="J104" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I104&lt;&gt;"","IO_LOC """&amp;I104&amp;""" "&amp;D104&amp;";", "")</f>
         <v>IO_LOC "mipi_d_p[3]" A5;</v>
       </c>
     </row>
@@ -5487,7 +5490,7 @@
         <v>325</v>
       </c>
       <c r="J105" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I105&lt;&gt;"","IO_LOC """&amp;I105&amp;""" "&amp;D105&amp;";", "")</f>
         <v>IO_LOC "mipi_gpio[0]" A1;</v>
       </c>
     </row>
@@ -5518,7 +5521,7 @@
         <v>326</v>
       </c>
       <c r="J106" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I106&lt;&gt;"","IO_LOC """&amp;I106&amp;""" "&amp;D106&amp;";", "")</f>
         <v>IO_LOC "mipi_gpio[1]" E3;</v>
       </c>
     </row>
@@ -5549,7 +5552,7 @@
         <v>302</v>
       </c>
       <c r="J107" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I107&lt;&gt;"","IO_LOC """&amp;I107&amp;""" "&amp;D107&amp;";", "")</f>
         <v>IO_LOC "mipi_pwr_en" G10;</v>
       </c>
     </row>
@@ -5580,7 +5583,7 @@
         <v>303</v>
       </c>
       <c r="J108" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I108&lt;&gt;"","IO_LOC """&amp;I108&amp;""" "&amp;D108&amp;";", "")</f>
         <v>IO_LOC "mipi_scl" D11;</v>
       </c>
     </row>
@@ -5611,7 +5614,7 @@
         <v>304</v>
       </c>
       <c r="J109" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I109&lt;&gt;"","IO_LOC """&amp;I109&amp;""" "&amp;D109&amp;";", "")</f>
         <v>IO_LOC "mipi_sda" D10;</v>
       </c>
     </row>
@@ -5644,7 +5647,7 @@
         <v>317</v>
       </c>
       <c r="J110" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I110&lt;&gt;"","IO_LOC """&amp;I110&amp;""" "&amp;D110&amp;";", "")</f>
         <v>IO_LOC "pmod[0]" F2;</v>
       </c>
     </row>
@@ -5677,7 +5680,7 @@
         <v>318</v>
       </c>
       <c r="J111" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I111&lt;&gt;"","IO_LOC """&amp;I111&amp;""" "&amp;D111&amp;";", "")</f>
         <v>IO_LOC "pmod[1]" F1;</v>
       </c>
     </row>
@@ -5708,7 +5711,7 @@
         <v>319</v>
       </c>
       <c r="J112" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I112&lt;&gt;"","IO_LOC """&amp;I112&amp;""" "&amp;D112&amp;";", "")</f>
         <v>IO_LOC "pmod[2]" B2;</v>
       </c>
     </row>
@@ -5739,7 +5742,7 @@
         <v>320</v>
       </c>
       <c r="J113" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I113&lt;&gt;"","IO_LOC """&amp;I113&amp;""" "&amp;D113&amp;";", "")</f>
         <v>IO_LOC "pmod[3]" C2;</v>
       </c>
     </row>
@@ -5772,7 +5775,7 @@
         <v>321</v>
       </c>
       <c r="J114" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I114&lt;&gt;"","IO_LOC """&amp;I114&amp;""" "&amp;D114&amp;";", "")</f>
         <v>IO_LOC "pmod[4]" E1;</v>
       </c>
     </row>
@@ -5803,7 +5806,7 @@
         <v>322</v>
       </c>
       <c r="J115" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I115&lt;&gt;"","IO_LOC """&amp;I115&amp;""" "&amp;D115&amp;";", "")</f>
         <v>IO_LOC "pmod[5]" D1;</v>
       </c>
     </row>
@@ -5834,7 +5837,7 @@
         <v>324</v>
       </c>
       <c r="J116" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I116&lt;&gt;"","IO_LOC """&amp;I116&amp;""" "&amp;D116&amp;";", "")</f>
         <v>IO_LOC "pmod[6]" B3;</v>
       </c>
     </row>
@@ -5865,25 +5868,25 @@
         <v>323</v>
       </c>
       <c r="J117" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I117&lt;&gt;"","IO_LOC """&amp;I117&amp;""" "&amp;D117&amp;";", "")</f>
         <v>IO_LOC "pmod[7]" C3;</v>
       </c>
     </row>
     <row r="118" spans="1:10">
       <c r="A118" s="3">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B118" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C118" s="4">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="F118" s="4">
         <v>6</v>
@@ -5893,28 +5896,28 @@
         <v>1.8</v>
       </c>
       <c r="I118" s="3" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="J118" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>IO_LOC "push_sw[0]" B11;</v>
+        <f>IF(I118&lt;&gt;"","IO_LOC """&amp;I118&amp;""" "&amp;D118&amp;";", "")</f>
+        <v>IO_LOC "push_sw[0]" B10;</v>
       </c>
     </row>
     <row r="119" spans="1:10">
       <c r="A119" s="3">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B119" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C119" s="4">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="F119" s="4">
         <v>6</v>
@@ -5924,11 +5927,11 @@
         <v>1.8</v>
       </c>
       <c r="I119" s="3" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="J119" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>IO_LOC "push_sw[1]" B10;</v>
+        <f>IF(I119&lt;&gt;"","IO_LOC """&amp;I119&amp;""" "&amp;D119&amp;";", "")</f>
+        <v>IO_LOC "push_sw[1]" B11;</v>
       </c>
     </row>
     <row r="120" spans="1:10">
@@ -5955,10 +5958,10 @@
         <v>3.3</v>
       </c>
       <c r="I120" s="3" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="J120" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I120&lt;&gt;"","IO_LOC """&amp;I120&amp;""" "&amp;D120&amp;";", "")</f>
         <v>IO_LOC "test[0]" E8;</v>
       </c>
     </row>
@@ -5986,10 +5989,10 @@
         <v>3.3</v>
       </c>
       <c r="I121" s="3" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="J121" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I121&lt;&gt;"","IO_LOC """&amp;I121&amp;""" "&amp;D121&amp;";", "")</f>
         <v>IO_LOC "test[1]" D7;</v>
       </c>
     </row>
@@ -6012,7 +6015,7 @@
       <c r="H122" s="3"/>
       <c r="I122" s="3"/>
       <c r="J122" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(I122&lt;&gt;"","IO_LOC """&amp;I122&amp;""" "&amp;D122&amp;";", "")</f>
         <v/>
       </c>
     </row>

</xml_diff>